<commit_message>
Delete multiple Stata scripts related to variable harmonization for education, ethnicity, RUC, and self-employment from the informal economy analysis. These scripts included harmonization processes for various demographic and economic variables spanning from 1990 to 2025.
</commit_message>
<xml_diff>
--- a/Dashboards/data/Data final/empleo/pobreza/pobreza_evolucion.xlsx
+++ b/Dashboards/data/Data final/empleo/pobreza/pobreza_evolucion.xlsx
@@ -336,10 +336,10 @@
         <v>2</v>
       </c>
       <c r="C19" s="1">
-        <v>0.29595917463302612</v>
+        <v>0.27703547477722168</v>
       </c>
       <c r="D19" s="1">
-        <v>29.595916748046875</v>
+        <v>27.703548431396484</v>
       </c>
     </row>
     <row r="20">
@@ -350,10 +350,10 @@
         <v>2</v>
       </c>
       <c r="C20" s="1">
-        <v>0.26901325583457947</v>
+        <v>0.2522730827331543</v>
       </c>
       <c r="D20" s="1">
-        <v>26.901325225830078</v>
+        <v>25.22730827331543</v>
       </c>
     </row>
     <row r="21">
@@ -364,10 +364,10 @@
         <v>2</v>
       </c>
       <c r="C21" s="1">
-        <v>0.2695763111114502</v>
+        <v>0.26023355126380921</v>
       </c>
       <c r="D21" s="1">
-        <v>26.957630157470703</v>
+        <v>26.023355484008789</v>
       </c>
     </row>
     <row r="22">
@@ -378,10 +378,10 @@
         <v>2</v>
       </c>
       <c r="C22" s="1">
-        <v>0.27970606088638306</v>
+        <v>0.27994614839553833</v>
       </c>
       <c r="D22" s="1">
-        <v>27.970605850219727</v>
+        <v>27.99461555480957</v>
       </c>
     </row>
     <row r="23">
@@ -392,10 +392,10 @@
         <v>2</v>
       </c>
       <c r="C23" s="1">
-        <v>0.2347552627325058</v>
+        <v>0.21370954811573029</v>
       </c>
       <c r="D23" s="1">
-        <v>23.475526809692383</v>
+        <v>21.370954513549805</v>
       </c>
     </row>
   </sheetData>

</xml_diff>